<commit_message>
Balanço 9.10 (marcos 1–4, commit intermédio): registo de riscos com critérios v1 (#4 Baixo, #7 Médio provisório, #2 Crítico exceção didática, novos #9 capacidade Alto e #10 alertas fora do SIEM Médio), Declaração (A.5.17/A.8.9 parciais, A.8.6 e A.8.15 novos), mapa MITRE, hardening-baseline pt.8, READMEs EN/PT com a Fase 9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/registo-riscos.xlsx
+++ b/registo-riscos.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -78,8 +78,13 @@
       <i val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +121,21 @@
         <bgColor rgb="FFD0D0D0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFE699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -151,7 +171,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -235,6 +255,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -547,7 +579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="14" min="1" max="1"/>
@@ -661,7 +693,7 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>Contenção ao nível do host (iptables na VM alvo, porque o segmento é L2 flat e uma regra no firewall perimetral não teria efeito); FTP anónimo passou a só-leitura; execução de PHP desativada na pasta de upload</t>
+          <t>Contenção ao nível do host (iptables na VM alvo, porque o segmento é L2 flat e uma regra no firewall perimetral não teria efeito); FTP anónimo passou a só-leitura; execução de PHP desativada na pasta de upload || Balanço 9.10 (20/10/2026): desde a 9.7 a Kali está na DMZ e a contenção no gateway passou a funcionar entre atacante e alvo (#127) — o texto "segmento L2 flat" deixou de se aplicar a este fluxo. Recusa do envio anónimo reconfirmada a partir da DMZ (550 e nada no disco, #129). Fragilidade adicional: /srv/ftp/upload continua 777 (enfraquece a defesa em profundidade e engana o nmap) — correção PLANEADA para a Fase 10 (não é aceitação formal). Por verificar na Fase 10: todos os caminhos de escrita anónima no servidor, incluindo a partilha Samba "publico" da #64 (escrita anónima não testada desde a Fase 4 — hipótese, não condição confirmada). Classificação mantida. Ainda não confrontado com os critérios v1 (Fase 10).</t>
         </is>
       </c>
       <c r="H2" s="18" t="n">
@@ -677,7 +709,7 @@
       </c>
       <c r="K2" s="17" t="inlineStr">
         <is>
-          <t>Entrada #104 — playbook de resposta a incidentes completo (deteção → triagem → contenção → erradicação → recuperação), 4 web shells encontradas e removidas</t>
+          <t>Entrada #104 — playbook de resposta a incidentes completo (deteção → triagem → contenção → erradicação → recuperação), 4 web shells encontradas e removidas; #127 (segmentação); #129 (reteste FTP, pasta 777)</t>
         </is>
       </c>
       <c r="L2" s="17" t="inlineStr">
@@ -715,7 +747,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>Nenhum — risco aceite conscientemente (decisão documentada no hardening-baseline, ponto 8), para manter a técnica reproduzível como exercício didático; gMSA identificado como a correção real fora de um lab</t>
+          <t>Exceção didática aceite. Classificação mantida em Crítico (3×3) por coerência com o contexto de avaliação da Fase 8 (organização fictícia, #107): nessa organização, svc_sql e svc_legacy seriam contas de serviço de produção, alcançáveis por qualquer conta de domínio no segmento Interno (plano). A classificação é sustentada pela matriz P×I (probabilidade alta: basta uma conta de domínio no Interno plano; impacto alto: contas de serviço do DC), não pelo contexto didático. As duas contas mantêm-se vulneráveis de propósito para preservar as demonstrações de Kerberoasting (svc_sql, #91) e AS-REP Roasting (svc_legacy, sem pré-autenticação, #92). Esta aceitação é específica do laboratório didático e não deve ser transposta para uma organização real sem uma avaliação formal do risco, das medidas de mitigação e da autoridade competente para o aceitar. Controlos compensatórios (detetivos): regra 100011 (Kerberoasting, TGS RC4, nível 10, #95) e regras 100010/100012 (AS-REP, #93/#94) — validadas nas Fases 6–7, não reverificadas na Fase 9; reduzem potencialmente o tempo até à deteção, não eliminam a vulnerabilidade nem impedem o ataque. Redução de exposição: desde a 9.7 a Kali (DMZ) não alcança o DC (política B, #127); não elimina o risco, porque o Interno é plano. Correção demonstrada noutras contas: gMSA svc_gmsa01 (#119) e svc_gmsa02 com grupo próprio (#123) — não altera svc_sql nem svc_legacy. Dono: Pedro. Aceitação: 2026-09-25 (hardening-baseline, ponto 8); reconfirmada 2026-10-20 (balanço 9.10). A reconfirmação de 20/10/2026 mantém a aceitação do risco no contexto didático, mas não constitui uma nova validação técnica das regras de deteção. Condição de revisão: quando a demonstração deixar de ser necessária, ou no encerramento do lab → corrigir (gMSA ou password longa e aleatória; ativar pré-autenticação Kerberos na svc_legacy) ou remover as contas. Reverificar as regras 100011/100010 na Fase 10. A migração "numa sessão própria" referida na #125 fica dependente desta condição.</t>
         </is>
       </c>
       <c r="H3" s="18" t="n">
@@ -731,7 +763,7 @@
       </c>
       <c r="K3" s="17" t="inlineStr">
         <is>
-          <t>Fase 6 (Kerberoasting/AS-REP Roasting); hardening-baseline.md, ponto 8</t>
+          <t>Fase 6 (#91, #92); regras #93–#95; hardening-baseline.md, ponto 8; gMSA #119, #123; #125; segmentação #127; balanço 9.10</t>
         </is>
       </c>
       <c r="L3" s="17" t="inlineStr">
@@ -823,23 +855,23 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Corrigido reativamente nesta sessão (docker restart) após deteção manual por nmap; sem controlo preventivo ou deteção automática ainda implementada</t>
+          <t>Balanço 9.10 (20/10/2026), critérios v1: controlo preventivo (o contentor recupera sozinho depois de um encerramento não limpo) e detetivo (healthcheck a cada minuto + alerta no Wazuh) provados com a mesma falha da #108 — deteta, regista, recupera, alerta (#124, 14/10/2026). Residual P1 (condições que limitam a ocorrência) × I2 (interrupção recuperável) = Baixo. Limitações: caminho AVISO-DOCKER/FALHA-DOCKER não testado ao vivo; o healthcheck corre dentro da própria VM (a VM inteira em baixo não é detetada); janela até ~2 min entre a queda e a recuperação; Apache 8080 fora do âmbito. Controlo testado uma vez — reverificar na Fase 10. (Antes: corrigido reativamente na #108, sem controlo.)</t>
         </is>
       </c>
       <c r="H5" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="J5" s="20" t="inlineStr">
-        <is>
-          <t>Médio</t>
+      <c r="J5" s="29" t="inlineStr">
+        <is>
+          <t>Baixo</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t>Entrada #108 — verificação ao vivo, Sessão 8.1</t>
+          <t>Entrada #108 — verificação ao vivo, Sessão 8.1; Entrada #124 (Sessão 9.4)</t>
         </is>
       </c>
       <c r="L5" s="17" t="inlineStr">
@@ -877,7 +909,7 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>Nenhum controlo de encriptação aplicado a estes fluxos. Aceite porque o lab é de teste e não tem dados pessoais reais de clientes. Numa organização real o tratamento seria HTTPS e SFTP/FTPS. Revisão se o lab passar a conter dados reais ou se for feita uma sessão sobre encriptação do tráfego interno.</t>
+          <t>Nenhum controlo de encriptação aplicado a estes fluxos. Aceite porque o lab é de teste e não tem dados pessoais reais de clientes. Numa organização real o tratamento seria HTTPS e SFTP/FTPS. Revisão se o lab passar a conter dados reais ou se for feita uma sessão sobre encriptação do tráfego interno. || Balanço 9.10 (20/10/2026): evidência nova — o nmap confirma FTP em texto limpo ("Control/Data connections will be plain text", #129). Sem alteração de nível. Ainda não confrontado com os critérios v1 (Fase 10).</t>
         </is>
       </c>
       <c r="H6" s="18" t="n">
@@ -893,7 +925,7 @@
       </c>
       <c r="K6" s="17" t="inlineStr">
         <is>
-          <t>Entrada #104 (FTP), Entrada #108 (HTTP, DVWA); revisto na Sessão 8.7 (a Entrada #97 não é evidência deste risco: mostra o envenenamento LLMNR do risco #3)</t>
+          <t>Entrada #104 (FTP), Entrada #108 (HTTP, DVWA); revisto na Sessão 8.7 (a Entrada #97 não é evidência deste risco: mostra o envenenamento LLMNR do risco #3); #129</t>
         </is>
       </c>
       <c r="L6" s="17" t="inlineStr">
@@ -931,7 +963,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Nenhum — risco aceite conscientemente e documentado (hardening-baseline, ponto 9; nota de limitação no mapa de cobertura MITRE ATT&amp;CK)</t>
+          <t>Nenhum — risco aceite conscientemente e documentado (hardening-baseline, ponto 9; nota de limitação no mapa de cobertura MITRE ATT&amp;CK) || Balanço 9.10 (20/10/2026): o próprio SIEM também está desatualizado — VM Wazuh com 46 atualizações disponíveis e reinício pendente (#129). Sem alteração de nível. Ainda não confrontado com os critérios v1 (Fase 10).</t>
         </is>
       </c>
       <c r="H7" s="18" t="n">
@@ -947,7 +979,7 @@
       </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
-          <t>hardening-baseline.md, ponto 9; mapa-cobertura-mitre-attack.md; Entrada #126 (scan nmap --script vuln: Apache 2.4.25 confirmado)</t>
+          <t>hardening-baseline.md, ponto 9; mapa-cobertura-mitre-attack.md; Entrada #126 (scan nmap --script vuln: Apache 2.4.25 confirmado); #129 (Wazuh)</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">
@@ -985,7 +1017,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>Mapa de cobertura corrigido para refletir com precisão que é um alerta enganador, não deteção real; nenhuma regra nova criada ainda para a técnica em si</t>
+          <t>Balanço 9.10 (20/10/2026), critérios v1: regra dedicada 100021 (nível 10, "Enumeração massiva do AD (padrão BloodHound)"), validada de ponta a ponta com teste contrário (#120, 08/10/2026). Cobre a enumeração RÁPIDA (200+ leituras em 30 s); NÃO cobre a enumeração lenta — bypass conhecido e documentado na própria #120, em que só aparecem os alertas de fábrica 92652/92657 (que continuam a disparar ao lado). Residual P2 (cenário plausível; o controlo não cobre a variante lenta) × I2 (redução relevante da capacidade de deteção) = Médio, PROVISÓRIO. Nota: a 1.ª proposta do balanço (baixar para Baixo) foi revista ao aplicar os critérios v1. Trabalho futuro (Fase 10): teste de enumeração lenta e eventual correção da regra.</t>
         </is>
       </c>
       <c r="H8" s="18" t="n">
@@ -994,14 +1026,14 @@
       <c r="I8" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="J8" s="20" t="inlineStr">
+      <c r="J8" s="30" t="inlineStr">
         <is>
           <t>Médio</t>
         </is>
       </c>
       <c r="K8" s="17" t="inlineStr">
         <is>
-          <t>Entrada #90 — threat hunting proativo, Fase 7</t>
+          <t>Entrada #90 — threat hunting proativo, Fase 7; Entrada #120 (Sessão 9.2)</t>
         </is>
       </c>
       <c r="L8" s="17" t="inlineStr">
@@ -1039,7 +1071,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal.</t>
+          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal. || Balanço 9.10 (20/10/2026): observação df -h — /home 89%, /mnt/VMs 80% (69% na #115), / 90%. Gatilho de revisão (/home ou /mnt/VMs acima de 90%) NÃO atingido (/home perto). O risco de capacidade passa a ter linha própria (#9); este risco continua a ser o de não conseguir recuperar. Ainda não confrontado com os critérios v1 (Fase 10).</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
@@ -1055,12 +1087,120 @@
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7</t>
+          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7; balanço 9.10 (df -h, 20/10/2026)</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
         <is>
           <t>ISO 27001 A.8.13; NIS2 Art.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="150" customHeight="1" s="15">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>Máquina física do lab (discos do Mint: /, /home, /mnt/VMs) e todas as VMs</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Esgotamento do espaço em disco: o VMware pausa ou pára as VMs, os snapshots falham ou ficam inconsistentes, o Mint deixa de conseguir atualizar</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Discos partilhados entre o lab e a formação; snapshots e cópias crescem sem política de snapshots nem limites de utilização; sem alerta formal</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>Nenhum controlo formal (só os alertas de espaço do projeto de hardening do PC). Balanço 9.10 (20/10/2026), critérios v1: P3 — ocorrência anterior relevante em condições comparáveis (#120: /home a 100%, VMware pausou as VMs) e utilização alta e a subir (/ 90%, /home 89%, /mnt/VMs 69%→80%), sem controlos eficazes; I2 — interrupção significativa mas recuperável, sem perda de dados demonstrada. A causa da subida do /mnt/VMs (snapshots da Fase 9?) é hipótese não verificada. Distinto do risco #8 (cópias de segurança). Tratamento: mitigar. Condição de revisão: definir política de snapshots, estabelecer limites de utilização e verificar a evolução dos discos ANTES de iniciar a Fase 10. Não apagar ficheiros nem snapshots sem primeiro identificar o que ocupa o espaço.</t>
+        </is>
+      </c>
+      <c r="H10" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="31" t="inlineStr">
+        <is>
+          <t>Alto</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="inlineStr">
+        <is>
+          <t>Entrada #120 (incidente de capacidade); #119–#125 (pedidos de política de snapshots); balanço 9.10 (df -h, 20/10/2026)</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>ISO 27001 A.8.6 (gestão da capacidade), A.8.13; NIS2 Art.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="150" customHeight="1" s="15">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>Deteção (Wazuh + Suricata no OPNsense)</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Ataque de rede detetado pelo IDS mas não visto pelo analista, que trabalha no SIEM — deteção tardia ou nenhuma</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Não existe integração Suricata → Wazuh: nenhum agente no OPNsense, o Wazuh não aceita syslog (só 1514/secure); os alertas ficam só no OPNsense, que ninguém consulta por rotina</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="G11" s="17" t="inlineStr">
+        <is>
+          <t>Nenhum (os agentes Wazuh nas VMs cobrem parte dos comportamentos, mas não substituem a visibilidade de rede). Balanço 9.10 (20/10/2026), critérios v1: P2 — exposição persistente, mas sem ameaça concreta demonstrada; o alerta existir no OPNsense NÃO baixa a probabilidade de deteção tardia. I2 — redução relevante da capacidade de deteção. Médio, PROVISÓRIO: impacto avaliado sobre a cobertura verificada (o Suricata só tem provado o reconhecimento — scans nmap); pode estar subavaliado. Gatilho de reclassificação: se na Fase 10 o Suricata detetar ataques à aplicação (ex.: SQLi, invisível no Wazuh — mapa MITRE linha 1) contra a "app + BD clientes" (C/I Alta, #108) → I3 → Alto. Tratamento: mitigar na Fase 10 (integração + verificação contínua de que os eventos continuam a chegar).</t>
+        </is>
+      </c>
+      <c r="H11" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t>Médio</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
+        <is>
+          <t>Entrada #129 (Sessão 9.9: três provas da inexistência da integração); pressuposto da #117 corrigido</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>ISO 27001 A.8.15, A.8.16</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="14" min="1" max="1"/>
@@ -1180,6 +1320,76 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>Critérios v1 (balanço 9.10, 20/10/2026) — operacionais do lab, não escala universal da ISO 27001:</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
+        <is>
+          <t>Probabilidade INERENTE: avalia-se só pela exposição e ameaça. Probabilidade RESIDUAL: considera os controlos existentes e a evidência da sua eficácia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
+        <is>
+          <t>I1 Baixo — consequências limitadas para a confidencialidade, integridade, disponibilidade ou deteção, com recuperação simples.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="28" t="inlineStr">
+        <is>
+          <t>I2 Médio — comprometimento significativo, interrupção recuperável ou redução relevante da capacidade de deteção, sem consequências graves demonstradas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="28" t="inlineStr">
+        <is>
+          <t>I3 Alto — exposição relevante de informação sensível, comprometimento grave, interrupção prolongada ou perda substancial da capacidade de detetar ataques.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>P1 Baixa — cenário pouco provável, considerando a exposição e a ameaça, com condições que limitam a sua ocorrência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="28" t="inlineStr">
+        <is>
+          <t>P2 Média — cenário plausível, dada a exposição e a ameaça, sem evidência suficiente para P1 ou P3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="28" t="inlineStr">
+        <is>
+          <t>P3 Alta — ocorrência anterior relevante em condições comparáveis, ou exposição persistente associada a uma ameaça concreta e a condições que favorecem a ocorrência, sem controlos eficazes demonstrados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="28" t="inlineStr">
+        <is>
+          <t>Histórico: a 1.ª versão do P3 ("exposição persistente, sem controlos") foi rejeitada por elevar artificialmente quase todos os riscos do lab; revista e reaplicada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>Aplicados aos riscos #4, #7, #9 e #10. Os riscos #1, #2, #3, #5, #6 e #8 ainda NÃO foram confrontados com estes critérios (reavaliação na Fase 10).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Sessão 9.10: balanço e fecho da Fase 9 — Entrada #130, guia de estudo da Fase 9, risco #4 corretivo (P2×I1), #2 avaliação vs aceitação separadas, syslog "não configurado" no #10, lista para a Fase 10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/registo-riscos.xlsx
+++ b/registo-riscos.xlsx
@@ -747,7 +747,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>Exceção didática aceite. Classificação mantida em Crítico (3×3) por coerência com o contexto de avaliação da Fase 8 (organização fictícia, #107): nessa organização, svc_sql e svc_legacy seriam contas de serviço de produção, alcançáveis por qualquer conta de domínio no segmento Interno (plano). A classificação é sustentada pela matriz P×I (probabilidade alta: basta uma conta de domínio no Interno plano; impacto alto: contas de serviço do DC), não pelo contexto didático. As duas contas mantêm-se vulneráveis de propósito para preservar as demonstrações de Kerberoasting (svc_sql, #91) e AS-REP Roasting (svc_legacy, sem pré-autenticação, #92). Esta aceitação é específica do laboratório didático e não deve ser transposta para uma organização real sem uma avaliação formal do risco, das medidas de mitigação e da autoridade competente para o aceitar. Controlos compensatórios (detetivos): regra 100011 (Kerberoasting, TGS RC4, nível 10, #95) e regras 100010/100012 (AS-REP, #93/#94) — validadas nas Fases 6–7, não reverificadas na Fase 9; reduzem potencialmente o tempo até à deteção, não eliminam a vulnerabilidade nem impedem o ataque. Redução de exposição: desde a 9.7 a Kali (DMZ) não alcança o DC (política B, #127); não elimina o risco, porque o Interno é plano. Correção demonstrada noutras contas: gMSA svc_gmsa01 (#119) e svc_gmsa02 com grupo próprio (#123) — não altera svc_sql nem svc_legacy. Dono: Pedro. Aceitação: 2026-09-25 (hardening-baseline, ponto 8); reconfirmada 2026-10-20 (balanço 9.10). A reconfirmação de 20/10/2026 mantém a aceitação do risco no contexto didático, mas não constitui uma nova validação técnica das regras de deteção. Condição de revisão: quando a demonstração deixar de ser necessária, ou no encerramento do lab → corrigir (gMSA ou password longa e aleatória; ativar pré-autenticação Kerberos na svc_legacy) ou remover as contas. Reverificar as regras 100011/100010 na Fase 10. A migração "numa sessão própria" referida na #125 fica dependente desta condição.</t>
+          <t>Exceção didática aceite. Classificação Crítica (3×3) herdada da Fase 8 (contexto da organização fictícia, #107) e reconfirmada pelo raciocínio de probabilidade e impacto; ainda NÃO confrontada com os critérios v1 (reavaliação na Fase 10). A decisão de aceitação é separada da avaliação: aceita-se o risco tal como está classificado, por razão didática. Contexto: nessa organização, svc_sql e svc_legacy seriam contas de serviço de produção, alcançáveis por qualquer conta de domínio no segmento Interno (plano). Raciocínio da classificação: probabilidade alta (basta uma conta de domínio no Interno plano); impacto alto (contas de serviço do DC) — não o contexto didático. As duas contas mantêm-se vulneráveis de propósito para preservar as demonstrações de Kerberoasting (svc_sql, #91) e AS-REP Roasting (svc_legacy, sem pré-autenticação, #92). Esta aceitação é específica do laboratório didático e não deve ser transposta para uma organização real sem uma avaliação formal do risco, das medidas de mitigação e da autoridade competente para o aceitar. Controlos compensatórios (detetivos): regra 100011 (Kerberoasting, TGS RC4, nível 10, #95) e regras 100010/100012 (AS-REP, #93/#94) — validadas nas Fases 6–7, não reverificadas na Fase 9; reduzem potencialmente o tempo até à deteção, não eliminam a vulnerabilidade nem impedem o ataque. Redução de exposição: desde a 9.7 a Kali (DMZ) não alcança o DC (política B, #127); não elimina o risco, porque o Interno é plano. Correção demonstrada noutras contas: gMSA svc_gmsa01 (#119) e svc_gmsa02 com grupo próprio (#123) — não altera svc_sql nem svc_legacy. Dono: Pedro. Aceitação: 2026-09-25 (hardening-baseline, ponto 8); reconfirmada 2026-10-20 (balanço 9.10). A reconfirmação de 20/10/2026 mantém a aceitação do risco no contexto didático, mas não constitui uma nova validação técnica das regras de deteção. Condição de revisão: quando a demonstração deixar de ser necessária, ou no encerramento do lab → corrigir (gMSA ou password longa e aleatória; ativar pré-autenticação Kerberos na svc_legacy) ou remover as contas. Reverificar as regras 100011/100010 na Fase 10. A migração "numa sessão própria" referida na #125 fica dependente desta condição.</t>
         </is>
       </c>
       <c r="H3" s="18" t="n">
@@ -855,14 +855,14 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Balanço 9.10 (20/10/2026), critérios v1: controlo preventivo (o contentor recupera sozinho depois de um encerramento não limpo) e detetivo (healthcheck a cada minuto + alerta no Wazuh) provados com a mesma falha da #108 — deteta, regista, recupera, alerta (#124, 14/10/2026). Residual P1 (condições que limitam a ocorrência) × I2 (interrupção recuperável) = Baixo. Limitações: caminho AVISO-DOCKER/FALHA-DOCKER não testado ao vivo; o healthcheck corre dentro da própria VM (a VM inteira em baixo não é detetada); janela até ~2 min entre a queda e a recuperação; Apache 8080 fora do âmbito. Controlo testado uma vez — reverificar na Fase 10. (Antes: corrigido reativamente na #108, sem controlo.)</t>
+          <t>Balanço 9.10 (20/10/2026), critérios v1: controlo CORRETIVO (recuperação automática: o script de saúde reinicia o contentor à 2.ª falha seguida) e DETETIVO (verificação a cada minuto + alerta no Wazuh), provados com a mesma falha da #108 — deteta, regista, recupera, alerta (#124, 14/10/2026). Nenhum dos dois impede a falha: o Apache pode continuar a morrer depois de um encerramento não limpo; reduzem a duração (até ~2 min) e garantem que a falha é vista. Residual: P2 (a falha continua possível) × I1 (consequências limitadas, recuperação simples e rápida, com alerta) = Baixo. Limitações: caminho AVISO-DOCKER/FALHA-DOCKER não testado ao vivo; o healthcheck corre dentro da própria VM (a VM inteira em baixo não é detetada); Apache 8080 fora do âmbito. Controlo testado uma vez — reverificar na Fase 10. (Antes: corrigido reativamente na #108, sem controlo. Nota: a #124 chamou "preventivo" à recuperação automática — classificação corrigida no balanço 9.10.)</t>
         </is>
       </c>
       <c r="H5" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="18" t="n">
         <v>1</v>
-      </c>
-      <c r="I5" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="J5" s="29" t="inlineStr">
         <is>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>Não existe integração Suricata → Wazuh: nenhum agente no OPNsense, o Wazuh não aceita syslog (só 1514/secure); os alertas ficam só no OPNsense, que ninguém consulta por rotina</t>
+          <t>Não existe integração Suricata → Wazuh: nenhum agente no OPNsense, sem receção de syslog configurada no Wazuh (só 1514/secure); os alertas ficam só no OPNsense, que ninguém consulta por rotina</t>
         </is>
       </c>
       <c r="D11" s="18" t="n">

</xml_diff>

<commit_message>
Entrada #134 (Sessão 10.0.4): critérios de aceitação no registo de riscos; riscos #8 (Alto, mitigar) e #9 (Alto, mantido) reavaliados; Declaração de Aplicabilidade atualizada — aprovado pelo Pedro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/registo-riscos.xlsx
+++ b/registo-riscos.xlsx
@@ -1062,32 +1062,32 @@
         <v>2</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal. || Balanço 9.10 (20/10/2026): observação df -h — /home 89%, /mnt/VMs 80% (69% na #115), / 90%. Gatilho de revisão (/home ou /mnt/VMs acima de 90%) NÃO atingido (/home perto). O risco de capacidade passa a ter linha própria (#9); este risco continua a ser o de não conseguir recuperar. Ainda não confrontado com os critérios v1 (Fase 10).</t>
+          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal. || Balanço 9.10 (20/10/2026): observação df -h — /home 89%, /mnt/VMs 80% (69% na #115), / 90%. Gatilho de revisão (/home ou /mnt/VMs acima de 90%) NÃO atingido (/home perto). O risco de capacidade passa a ter linha própria (#9); este risco continua a ser o de não conseguir recuperar. Ainda não confrontado com os critérios v1 (Fase 10). || Sessão 10.0.4 (26/10/2026): confrontado pela primeira vez com os critérios v1. Factos novos (#131, #132): nenhuma cópia independente das VMs confirmada (pasta BACKUP vazia; procura não exaustiva); os 14 snapshots identificados estão no mesmo disco das VMs e não são cópias; o Timeshift (35G no nvme) cobre só o sistema do Mint e a reposição nunca foi testada; / e /home estão no mesmo disco físico (sda), onde estão o DC, o Wazuh, o Windows 11 e o Servidor Vulnerável. P2 mantém-se: avaria plausível, sem perda de dados anterior (#114 e #120 não perderam dados); a ausência de proteção aumenta a exposição, não prova maior probabilidade. I2 → I3: a perda do sda causaria a indisponibilidade simultânea do DC e do Wazuh, com interrupção dos serviços do AD e da monitorização centralizada e perda potencial do histórico não guardado noutro local. [DEDUÇÃO] Reconstruir a partir da documentação (GitHub) levaria vários dias — estimativa, não tempo medido —, incompatível com o RTO de um dia aprovado na R6 da política (Entrada #133). Inerente e residual: P2 × I3 = Alto (sem cópias de segurança das VMs, coincidem; o GitHub é uma medida de recuperação da documentação, não uma cópia das VMs). Pela decisão 6, um risco Alto deixa de poder ser só aceite: tratamento passa a mitigar, através da R6 (cópias independentes do DC e do Wazuh; suporte por decidir). Prioridade: executar a R6 antes do 10.4 (alterações ao Wazuh); se não for possível, avançar só por decisão deliberada e registada. Revisão: após a criação, verificação e teste de reposição das cópias, ou se houver alteração material das condições (ex.: decisão sobre o disco, /home ou /mnt/VMs acima de 90%) — o gatilho desencadeia uma reavaliação, não uma alteração automática da classificação.</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
         <v>2</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J9" s="20" t="inlineStr">
         <is>
-          <t>Médio</t>
+          <t>Alto</t>
         </is>
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7; balanço 9.10 (df -h, 20/10/2026)</t>
+          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7; balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026)</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Nenhum controlo formal (só os alertas de espaço do projeto de hardening do PC). Balanço 9.10 (20/10/2026), critérios v1: P3 — ocorrência anterior relevante em condições comparáveis (#120: /home a 100%, VMware pausou as VMs) e utilização alta e a subir (/ 90%, /home 89%, /mnt/VMs 69%→80%), sem controlos eficazes; I2 — interrupção significativa mas recuperável, sem perda de dados demonstrada. A causa da subida do /mnt/VMs (snapshots da Fase 9?) é hipótese não verificada. Distinto do risco #8 (cópias de segurança). Tratamento: mitigar. Condição de revisão: definir política de snapshots, estabelecer limites de utilização e verificar a evolução dos discos ANTES de iniciar a Fase 10. Não apagar ficheiros nem snapshots sem primeiro identificar o que ocupa o espaço.</t>
+          <t>Nenhum controlo formal (só os alertas de espaço do projeto de hardening do PC). Balanço 9.10 (20/10/2026), critérios v1: P3 — ocorrência anterior relevante em condições comparáveis (#120: /home a 100%, VMware pausou as VMs) e utilização alta e a subir (/ 90%, /home 89%, /mnt/VMs 69%→80%), sem controlos eficazes; I2 — interrupção significativa mas recuperável, sem perda de dados demonstrada. A causa da subida do /mnt/VMs (snapshots da Fase 9?) é hipótese não verificada. Distinto do risco #8 (cópias de segurança). Tratamento: mitigar. Condição de revisão: definir política de snapshots, estabelecer limites de utilização e verificar a evolução dos discos ANTES de iniciar a Fase 10. Não apagar ficheiros nem snapshots sem primeiro identificar o que ocupa o espaço. || Sessão 10.0.4 (26/10/2026): política de snapshots, cópias e capacidade aprovada (Entrada #133, politicas/politica-snapshots-copias-capacidade.md), ainda não aplicada a nenhuma operação. Medição df -h (26/10): / 89%, /home 89%, /mnt/VMs 77%. A revisão exigida pela R5 para / e /home (acima de 85%) fica feita por análise e registo das medições; não resolve a capacidade. Critérios v1: P3 mantém-se (política escrita não é controlo eficaz demonstrado; condições comparáveis às da #120 — fundamentação do P3, não prova de que a causa atual é a mesma); I2 mantém-se. Residual mantém-se Alto; tratamento: mitigar. A R3 só se dá como aplicada quando as sete verificações forem feitas e documentadas para uma operação concreta. Revisão: após a primeira aplicação documentada da R5 e da R3, ou imediatamente se alguma partição ultrapassar 90% (o que desencadeia uma reavaliação, não uma remoção automática).</t>
         </is>
       </c>
       <c r="H10" s="18" t="n">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="K10" s="17" t="inlineStr">
         <is>
-          <t>Entrada #120 (incidente de capacidade); #119–#125 (pedidos de política de snapshots); balanço 9.10 (df -h, 20/10/2026)</t>
+          <t>Entrada #120 (incidente de capacidade); #119–#125 (pedidos de política de snapshots); balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026)</t>
         </is>
       </c>
       <c r="L10" s="17" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="14" min="1" max="1"/>
@@ -1390,6 +1390,48 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Critérios de aceitação do risco v1 (decisão 6 da proposta da Fase 10, aprovada a 23/10/2026; registados na Sessão 10.0.4, 26/10/2026):</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>O responsável pelo laboratório (o Pedro) decide sobre a aceitação do risco residual, com base na evidência recolhida, no impacto potencial e na eficácia dos controlos existentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="28" t="inlineStr">
+        <is>
+          <t>Baixo: pode ser aceite mediante registo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="28" t="inlineStr">
+        <is>
+          <t>Médio: exige justificação documentada e revisão definida (data ou condição).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Alto ou Crítico: exige tratamento, ou uma exceção temporária explicitamente justificada, delimitada e sujeita a revisão.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="28" t="inlineStr">
+        <is>
+          <t>A aceitação do risco não equivale à demonstração de que o controlo é eficaz, nem à eliminação do risco.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Fecho do bloco 10.0: Entrada #136 e revisão documental
- Registo: Entrada #136 (fecho do bloco 10.0)
- Registo de riscos: nota de revisão no risco #6 (evidência #135, #136)
- topologia-base e hardening-baseline: egress filtering limitado às quatro VMs com regras próprias
- Guia de acompanhamento: verificações e pendências atualizadas (fecho do bloco marcado num segundo commit)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/registo-riscos.xlsx
+++ b/registo-riscos.xlsx
@@ -963,7 +963,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>Nenhum — risco aceite conscientemente e documentado (hardening-baseline, ponto 9; nota de limitação no mapa de cobertura MITRE ATT&amp;CK) || Balanço 9.10 (20/10/2026): o próprio SIEM também está desatualizado — VM Wazuh com 46 atualizações disponíveis e reinício pendente (#129). Sem alteração de nível. Ainda não confrontado com os critérios v1 (Fase 10).</t>
+          <t>Nenhum — risco aceite conscientemente e documentado (hardening-baseline, ponto 9; nota de limitação no mapa de cobertura MITRE ATT&amp;CK) || Balanço 9.10 (20/10/2026): o próprio SIEM também está desatualizado — VM Wazuh com 46 atualizações disponíveis e reinício pendente (#129). Sem alteração de nível. Ainda não confrontado com os critérios v1 (Fase 10). || Sessão 10.0.5 (27/10/2026), fecho do bloco 10.0: confrontado com os critérios v1. P2 mantém-se (exploração plausível; lab sem exposição à internet; a exploração que ocorre no lab é a deliberada dos exercícios). I2 mantém-se (comprometimento significativo, recuperável). Classificação mantida: Médio, aceite. Pela decisão 6, um Médio aceite exige revisão definida. Revisão: no fecho da Fase 10; ou se alguma VM do lab passar a ter exposição fora da rede interna; ou se a decisão de manter estas VMs sem atualizações para os exercícios for alterada ou deixar de se justificar. Wazuh (#135): 30 atualizações listadas (lista de 20/10) e sem reinício pendente; não é uma das VMs deixadas sem atualizações de propósito (hardening-baseline, ponto 9) — a sua atualização está prevista para o início do 10.4, condicionada às cópias (R6).</t>
         </is>
       </c>
       <c r="H7" s="18" t="n">
@@ -979,7 +979,7 @@
       </c>
       <c r="K7" s="17" t="inlineStr">
         <is>
-          <t>hardening-baseline.md, ponto 9; mapa-cobertura-mitre-attack.md; Entrada #126 (scan nmap --script vuln: Apache 2.4.25 confirmado); #129 (Wazuh)</t>
+          <t>hardening-baseline.md, ponto 9; mapa-cobertura-mitre-attack.md; Entrada #126 (scan nmap --script vuln: Apache 2.4.25 confirmado); #129 (Wazuh); #135; #136</t>
         </is>
       </c>
       <c r="L7" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Entrada #137 (Sessão 10.1.1): medição R5 no início da sessão, remoção de cópias antigas do Timeshift, reavaliação dos riscos #8 e #9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lk2S9R4Pvx1JAK73UPgK7J
</commit_message>
<xml_diff>
--- a/registo-riscos.xlsx
+++ b/registo-riscos.xlsx
@@ -1071,7 +1071,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal. || Balanço 9.10 (20/10/2026): observação df -h — /home 89%, /mnt/VMs 80% (69% na #115), / 90%. Gatilho de revisão (/home ou /mnt/VMs acima de 90%) NÃO atingido (/home perto). O risco de capacidade passa a ter linha própria (#9); este risco continua a ser o de não conseguir recuperar. Ainda não confrontado com os critérios v1 (Fase 10). || Sessão 10.0.4 (26/10/2026): confrontado pela primeira vez com os critérios v1. Factos novos (#131, #132): nenhuma cópia independente das VMs confirmada (pasta BACKUP vazia; procura não exaustiva); os 14 snapshots identificados estão no mesmo disco das VMs e não são cópias; o Timeshift (35G no nvme) cobre só o sistema do Mint e a reposição nunca foi testada; / e /home estão no mesmo disco físico (sda), onde estão o DC, o Wazuh, o Windows 11 e o Servidor Vulnerável. P2 mantém-se: avaria plausível, sem perda de dados anterior (#114 e #120 não perderam dados); a ausência de proteção aumenta a exposição, não prova maior probabilidade. I2 → I3: a perda do sda causaria a indisponibilidade simultânea do DC e do Wazuh, com interrupção dos serviços do AD e da monitorização centralizada e perda potencial do histórico não guardado noutro local. [DEDUÇÃO] Reconstruir a partir da documentação (GitHub) levaria vários dias — estimativa, não tempo medido —, incompatível com o RTO de um dia aprovado na R6 da política (Entrada #133). Inerente e residual: P2 × I3 = Alto (sem cópias de segurança das VMs, coincidem; o GitHub é uma medida de recuperação da documentação, não uma cópia das VMs). Pela decisão 6, um risco Alto deixa de poder ser só aceite: tratamento passa a mitigar, através da R6 (cópias independentes do DC e do Wazuh; suporte por decidir). Prioridade: executar a R6 antes do 10.4 (alterações ao Wazuh); se não for possível, avançar só por decisão deliberada e registada. Revisão: após a criação, verificação e teste de reposição das cópias, ou se houver alteração material das condições (ex.: decisão sobre o disco, /home ou /mnt/VMs acima de 90%) — o gatilho desencadeia uma reavaliação, não uma alteração automática da classificação.</t>
+          <t>Nenhum para as VMs — risco aceite conscientemente (disco insuficiente; os discos servem também para o material da formação). Atenuante: a documentação do lab (registo, guias, scripts) está no GitHub e as VMs refazem-se a partir dela. Revisão se for comprado um disco externo ou se /home ou /mnt/VMs passarem de 90%; os alertas de espaço do projeto de hardening do PC funcionam como sinal. || Balanço 9.10 (20/10/2026): observação df -h — /home 89%, /mnt/VMs 80% (69% na #115), / 90%. Gatilho de revisão (/home ou /mnt/VMs acima de 90%) NÃO atingido (/home perto). O risco de capacidade passa a ter linha própria (#9); este risco continua a ser o de não conseguir recuperar. Ainda não confrontado com os critérios v1 (Fase 10). || Sessão 10.0.4 (26/10/2026): confrontado pela primeira vez com os critérios v1. Factos novos (#131, #132): nenhuma cópia independente das VMs confirmada (pasta BACKUP vazia; procura não exaustiva); os 14 snapshots identificados estão no mesmo disco das VMs e não são cópias; o Timeshift (35G no nvme) cobre só o sistema do Mint e a reposição nunca foi testada; / e /home estão no mesmo disco físico (sda), onde estão o DC, o Wazuh, o Windows 11 e o Servidor Vulnerável. P2 mantém-se: avaria plausível, sem perda de dados anterior (#114 e #120 não perderam dados); a ausência de proteção aumenta a exposição, não prova maior probabilidade. I2 → I3: a perda do sda causaria a indisponibilidade simultânea do DC e do Wazuh, com interrupção dos serviços do AD e da monitorização centralizada e perda potencial do histórico não guardado noutro local. [DEDUÇÃO] Reconstruir a partir da documentação (GitHub) levaria vários dias — estimativa, não tempo medido —, incompatível com o RTO de um dia aprovado na R6 da política (Entrada #133). Inerente e residual: P2 × I3 = Alto (sem cópias de segurança das VMs, coincidem; o GitHub é uma medida de recuperação da documentação, não uma cópia das VMs). Pela decisão 6, um risco Alto deixa de poder ser só aceite: tratamento passa a mitigar, através da R6 (cópias independentes do DC e do Wazuh; suporte por decidir). Prioridade: executar a R6 antes do 10.4 (alterações ao Wazuh); se não for possível, avançar só por decisão deliberada e registada. Revisão: após a criação, verificação e teste de reposição das cópias, ou se houver alteração material das condições (ex.: decisão sobre o disco, /home ou /mnt/VMs acima de 90%) — o gatilho desencadeia uma reavaliação, não uma alteração automática da classificação. || Sessão 10.1.1 (28/10/2026): reavaliação exigida pela R5 (`/home` acima de 90%). Sem evidência nova sobre as cópias: P2 e I3 mantêm-se. Classificação mantida: Alto (2×3), mitigar através da R6. Observado um disco externo ligado (`sdb1`, "TOSHIBA"), possível suporte para a R6; capacidade e conteúdo por verificar.</t>
         </is>
       </c>
       <c r="H9" s="18" t="n">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="K9" s="17" t="inlineStr">
         <is>
-          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7; balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026)</t>
+          <t>Entrada #115 — inventário de discos e do Timeshift (2026-09-30/10-01); decisão na Sessão 8.7; balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026); #137</t>
         </is>
       </c>
       <c r="L9" s="17" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Nenhum controlo formal (só os alertas de espaço do projeto de hardening do PC). Balanço 9.10 (20/10/2026), critérios v1: P3 — ocorrência anterior relevante em condições comparáveis (#120: /home a 100%, VMware pausou as VMs) e utilização alta e a subir (/ 90%, /home 89%, /mnt/VMs 69%→80%), sem controlos eficazes; I2 — interrupção significativa mas recuperável, sem perda de dados demonstrada. A causa da subida do /mnt/VMs (snapshots da Fase 9?) é hipótese não verificada. Distinto do risco #8 (cópias de segurança). Tratamento: mitigar. Condição de revisão: definir política de snapshots, estabelecer limites de utilização e verificar a evolução dos discos ANTES de iniciar a Fase 10. Não apagar ficheiros nem snapshots sem primeiro identificar o que ocupa o espaço. || Sessão 10.0.4 (26/10/2026): política de snapshots, cópias e capacidade aprovada (Entrada #133, politicas/politica-snapshots-copias-capacidade.md), ainda não aplicada a nenhuma operação. Medição df -h (26/10): / 89%, /home 89%, /mnt/VMs 77%. A revisão exigida pela R5 para / e /home (acima de 85%) fica feita por análise e registo das medições; não resolve a capacidade. Critérios v1: P3 mantém-se (política escrita não é controlo eficaz demonstrado; condições comparáveis às da #120 — fundamentação do P3, não prova de que a causa atual é a mesma); I2 mantém-se. Residual mantém-se Alto; tratamento: mitigar. A R3 só se dá como aplicada quando as sete verificações forem feitas e documentadas para uma operação concreta. Revisão: após a primeira aplicação documentada da R5 e da R3, ou imediatamente se alguma partição ultrapassar 90% (o que desencadeia uma reavaliação, não uma remoção automática).</t>
+          <t>Nenhum controlo formal (só os alertas de espaço do projeto de hardening do PC). Balanço 9.10 (20/10/2026), critérios v1: P3 — ocorrência anterior relevante em condições comparáveis (#120: /home a 100%, VMware pausou as VMs) e utilização alta e a subir (/ 90%, /home 89%, /mnt/VMs 69%→80%), sem controlos eficazes; I2 — interrupção significativa mas recuperável, sem perda de dados demonstrada. A causa da subida do /mnt/VMs (snapshots da Fase 9?) é hipótese não verificada. Distinto do risco #8 (cópias de segurança). Tratamento: mitigar. Condição de revisão: definir política de snapshots, estabelecer limites de utilização e verificar a evolução dos discos ANTES de iniciar a Fase 10. Não apagar ficheiros nem snapshots sem primeiro identificar o que ocupa o espaço. || Sessão 10.0.4 (26/10/2026): política de snapshots, cópias e capacidade aprovada (Entrada #133, politicas/politica-snapshots-copias-capacidade.md), ainda não aplicada a nenhuma operação. Medição df -h (26/10): / 89%, /home 89%, /mnt/VMs 77%. A revisão exigida pela R5 para / e /home (acima de 85%) fica feita por análise e registo das medições; não resolve a capacidade. Critérios v1: P3 mantém-se (política escrita não é controlo eficaz demonstrado; condições comparáveis às da #120 — fundamentação do P3, não prova de que a causa atual é a mesma); I2 mantém-se. Residual mantém-se Alto; tratamento: mitigar. A R3 só se dá como aplicada quando as sete verificações forem feitas e documentadas para uma operação concreta. Revisão: após a primeira aplicação documentada da R5 e da R3, ou imediatamente se alguma partição ultrapassar 90% (o que desencadeia uma reavaliação, não uma remoção automática). || Sessão 10.1.1 (28/10/2026): reavaliação exigida pela R5. `/home` medido a 90,74% no início da sessão (seis VMs ligadas), acima do limite de 90%; a condição de revisão deste risco verificou-se. Investigação só em leitura: 33G (`du -sh`, valor arredondado) numa localização antiga do Timeshift (`/home/timeshift`), com duas pastas de snapshot chamadas 2026-09-05_17-00-01 e 2026-09-06_17-00-01 (datas pelos nomes e pelas datas das pastas; conteúdo não inspecionado), fora da localização que o Timeshift gere (UUID do `nvme0n1p1`, `/mnt/VMs`). Removida por decisão do Pedro; `/home` passou de 90,77% para 82,65% (valores exatos, imediatamente antes e depois), com cerca de 32,5G libertados. A correspondência é forte, mas não permite atribuir toda a variação exclusivamente à remoção, dado que havia VMs em execução e o tamanho da pasta só foi medido de forma arredondada. As cópias ativas do Timeshift (27 e 28/10, em `/mnt/VMs`) foram listadas antes e depois; a sua existência foi confirmada, mas a integridade e a capacidade de reposição não foram testadas. P3 mantém-se: uma limpeza pontual não demonstra a eficácia do controlo. I2 mantém-se. Classificação mantida: Alto (3×2), mitigar. A revisão periódica do espaço em disco mantém-se como medida de mitigação, acompanhada no projeto de hardening do Mint.</t>
         </is>
       </c>
       <c r="H10" s="18" t="n">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="K10" s="17" t="inlineStr">
         <is>
-          <t>Entrada #120 (incidente de capacidade); #119–#125 (pedidos de política de snapshots); balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026)</t>
+          <t>Entrada #120 (incidente de capacidade); #119–#125 (pedidos de política de snapshots); balanço 9.10 (df -h, 20/10/2026); Sessão 10.0.4 (26/10/2026); #137</t>
         </is>
       </c>
       <c r="L10" s="17" t="inlineStr">

</xml_diff>